<commit_message>
Import approved LINE batch set_single636550441915908205
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B3_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B3_2026.xlsx
@@ -133,10 +133,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -168,10 +168,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -2449,7 +2449,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AE3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2547,10 +2547,36 @@
       <c r="AD2" t="str">
         <v>Used Young Coco</v>
       </c>
+      <c r="AE2" t="str">
+        <v>Source Note</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>14/10/2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C3">
+        <v>6821</v>
+      </c>
+      <c r="D3">
+        <v>5361</v>
+      </c>
+      <c r="E3">
+        <v>55</v>
+      </c>
+      <c r="G3">
+        <v>1460</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>LINE set_single636550441915908205 sha256:18fe5952773c | some cup counts were uncertain and were not written</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Import B3 sales Oct 2026 from Parn's Daily Shop Report photos (approved by Parn)
14 days, revenue 90599 (--day12=B12). 14/10 (LINE batch, 6821) unchanged.
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B3_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B3_2026.xlsx
@@ -133,10 +133,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -168,10 +168,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -2449,7 +2449,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2574,9 +2574,709 @@
         <v>LINE set_single636550441915908205 sha256:18fe5952773c | some cup counts were uncertain and were not written</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C4">
+        <v>4586</v>
+      </c>
+      <c r="D4">
+        <v>3654</v>
+      </c>
+      <c r="E4">
+        <v>55</v>
+      </c>
+      <c r="G4">
+        <v>932</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>16</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="L4">
+        <v>15</v>
+      </c>
+      <c r="M4">
+        <v>4</v>
+      </c>
+      <c r="O4">
+        <v>4</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="Q4">
+        <v>56</v>
+      </c>
+      <c r="AE4" t="str">
+        <v>Parn LINE photo 2a99558801b9 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Mangosteen Blended 8, Rambutan Blended 2, Mango Sticky Rice 1, Mango Sticky Rice (180) 1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C5">
+        <v>6786</v>
+      </c>
+      <c r="D5">
+        <v>4851</v>
+      </c>
+      <c r="E5">
+        <v>110</v>
+      </c>
+      <c r="G5">
+        <v>1935</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>17</v>
+      </c>
+      <c r="K5">
+        <v>12</v>
+      </c>
+      <c r="L5">
+        <v>10</v>
+      </c>
+      <c r="M5">
+        <v>8</v>
+      </c>
+      <c r="O5">
+        <v>8</v>
+      </c>
+      <c r="P5">
+        <v>7</v>
+      </c>
+      <c r="Q5">
+        <v>76</v>
+      </c>
+      <c r="AE5" t="str">
+        <v>Parn LINE photo 304767194108 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Mangosteen Lychee Blended 4, Mango Sticky Rice 2, Cold Pressed Mango Juice 3 | CHECK: items 6876 vs total sales 6786 (+90)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>03/10/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C6">
+        <v>6623</v>
+      </c>
+      <c r="D6">
+        <v>3899</v>
+      </c>
+      <c r="E6">
+        <v>55</v>
+      </c>
+      <c r="G6">
+        <v>2724</v>
+      </c>
+      <c r="H6">
+        <v>14</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>15</v>
+      </c>
+      <c r="K6">
+        <v>8</v>
+      </c>
+      <c r="L6">
+        <v>15</v>
+      </c>
+      <c r="M6">
+        <v>11</v>
+      </c>
+      <c r="O6">
+        <v>1</v>
+      </c>
+      <c r="P6">
+        <v>8</v>
+      </c>
+      <c r="Q6">
+        <v>80</v>
+      </c>
+      <c r="AE6" t="str">
+        <v>Parn LINE photo c4bc76799df9 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Mangosteen Blended 4, Mangosteen Lychee Blended 1, Volcano Mix Fruit 1, Mango Sticky Rice 1, Mango Sticky Rice (180) 1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>04/10/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C7">
+        <v>9583</v>
+      </c>
+      <c r="D7">
+        <v>6269</v>
+      </c>
+      <c r="E7">
+        <v>254</v>
+      </c>
+      <c r="G7">
+        <v>3314</v>
+      </c>
+      <c r="H7">
+        <v>15</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>29</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>31</v>
+      </c>
+      <c r="M7">
+        <v>11</v>
+      </c>
+      <c r="O7">
+        <v>8</v>
+      </c>
+      <c r="P7">
+        <v>5</v>
+      </c>
+      <c r="Q7">
+        <v>123</v>
+      </c>
+      <c r="AE7" t="str">
+        <v>Parn LINE photo 0167ca668ee7 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | exp incl. Condensed Milk 144 | not in fruit columns: Mangosteen Blended 1, Mangosteen Lychee Blended 4, Mango Sticky Rice 5, Mango Sticky Rice (180) 1, Pomegranate 4 | CHECK: items 9760 vs total sales 9583 (+177)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>05/10/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C8">
+        <v>4848</v>
+      </c>
+      <c r="D8">
+        <v>3083</v>
+      </c>
+      <c r="E8">
+        <v>251</v>
+      </c>
+      <c r="G8">
+        <v>1765</v>
+      </c>
+      <c r="H8">
+        <v>9</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>14</v>
+      </c>
+      <c r="K8">
+        <v>7</v>
+      </c>
+      <c r="L8">
+        <v>9</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+      <c r="O8">
+        <v>3</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8">
+        <v>51</v>
+      </c>
+      <c r="AE8" t="str">
+        <v>Parn LINE photo 95b4be4f1f66 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | exp incl. Meiji Milk 72, Falcon (2) 124 | not in fruit columns: Mangosteen Blended 1, Volcano Mix Fruit 1, Pomegranate 3 | CHECK: items 4847 vs total sales 4848 (-1)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>06/10/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C9">
+        <v>4280</v>
+      </c>
+      <c r="D9">
+        <v>3023</v>
+      </c>
+      <c r="E9">
+        <v>110</v>
+      </c>
+      <c r="G9">
+        <v>1257</v>
+      </c>
+      <c r="H9">
+        <v>4</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>10</v>
+      </c>
+      <c r="K9">
+        <v>2</v>
+      </c>
+      <c r="L9">
+        <v>19</v>
+      </c>
+      <c r="M9">
+        <v>7</v>
+      </c>
+      <c r="O9">
+        <v>3</v>
+      </c>
+      <c r="P9">
+        <v>3</v>
+      </c>
+      <c r="Q9">
+        <v>56</v>
+      </c>
+      <c r="AE9" t="str">
+        <v>Parn LINE photo 986ac49e9396 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Grape 3, Volcano Mix Fruit 2, Pear 2, Pomegranate 1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C10">
+        <v>4737</v>
+      </c>
+      <c r="D10">
+        <v>3407</v>
+      </c>
+      <c r="E10">
+        <v>55</v>
+      </c>
+      <c r="G10">
+        <v>1330</v>
+      </c>
+      <c r="H10">
+        <v>8</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>15</v>
+      </c>
+      <c r="K10">
+        <v>5</v>
+      </c>
+      <c r="L10">
+        <v>6</v>
+      </c>
+      <c r="M10">
+        <v>6</v>
+      </c>
+      <c r="O10">
+        <v>4</v>
+      </c>
+      <c r="P10">
+        <v>4</v>
+      </c>
+      <c r="Q10">
+        <v>58</v>
+      </c>
+      <c r="AE10" t="str">
+        <v>Parn LINE photo 6e3fa4cccd28 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Grape 3, Pear 1, Volcano Mix Fruit 1, Pomegranate 5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>08/10/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C11">
+        <v>6569</v>
+      </c>
+      <c r="D11">
+        <v>4377</v>
+      </c>
+      <c r="E11">
+        <v>55</v>
+      </c>
+      <c r="G11">
+        <v>2192</v>
+      </c>
+      <c r="H11">
+        <v>5</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>29</v>
+      </c>
+      <c r="K11">
+        <v>6</v>
+      </c>
+      <c r="L11">
+        <v>19</v>
+      </c>
+      <c r="M11">
+        <v>9</v>
+      </c>
+      <c r="O11">
+        <v>5</v>
+      </c>
+      <c r="P11">
+        <v>2</v>
+      </c>
+      <c r="Q11">
+        <v>87</v>
+      </c>
+      <c r="AE11" t="str">
+        <v>Parn LINE photo 280755341c77 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 2, Mangosteen Lychee Blended 6, Pear 1, Grape 3 | CHECK: items 6520 vs total sales 6569 (-49)</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C12">
+        <v>9383</v>
+      </c>
+      <c r="D12">
+        <v>6973</v>
+      </c>
+      <c r="E12">
+        <v>110</v>
+      </c>
+      <c r="G12">
+        <v>2410</v>
+      </c>
+      <c r="H12">
+        <v>17</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>24</v>
+      </c>
+      <c r="K12">
+        <v>14</v>
+      </c>
+      <c r="L12">
+        <v>15</v>
+      </c>
+      <c r="M12">
+        <v>8</v>
+      </c>
+      <c r="O12">
+        <v>14</v>
+      </c>
+      <c r="P12">
+        <v>5</v>
+      </c>
+      <c r="Q12">
+        <v>110</v>
+      </c>
+      <c r="AE12" t="str">
+        <v>Parn LINE photo 4714870e0a9d (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Pear 2, Grape 6, Pomegranate 3, Volcano Mix Fruit 1 | CHECK: items 9315 vs total sales 9383 (-68)</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>11/10/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C13">
+        <v>6874</v>
+      </c>
+      <c r="D13">
+        <v>4290</v>
+      </c>
+      <c r="E13">
+        <v>55</v>
+      </c>
+      <c r="G13">
+        <v>2584</v>
+      </c>
+      <c r="H13">
+        <v>15</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>19</v>
+      </c>
+      <c r="K13">
+        <v>9</v>
+      </c>
+      <c r="L13">
+        <v>16</v>
+      </c>
+      <c r="M13">
+        <v>8</v>
+      </c>
+      <c r="O13">
+        <v>8</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>87</v>
+      </c>
+      <c r="AE13" t="str">
+        <v>Parn LINE photo 413bb3937c75 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Pear 5, Mangosteen Lychee Blended 3, Pomegranate 3, Mango Sticky Rice (180) 1 | CHECK: items 6789 vs total sales 6874 (-85)</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C14">
+        <v>6118</v>
+      </c>
+      <c r="D14">
+        <v>4581</v>
+      </c>
+      <c r="E14">
+        <v>110</v>
+      </c>
+      <c r="G14">
+        <v>1537</v>
+      </c>
+      <c r="H14">
+        <v>7</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>13</v>
+      </c>
+      <c r="K14">
+        <v>11</v>
+      </c>
+      <c r="L14">
+        <v>15</v>
+      </c>
+      <c r="M14">
+        <v>4</v>
+      </c>
+      <c r="O14">
+        <v>6</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>71</v>
+      </c>
+      <c r="AE14" t="str">
+        <v>Parn LINE photo abc0ad7c829d (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Mangosteen Lychee Blended 4, Pomegranate 7, Grape 3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>13/10/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C15">
+        <v>8873</v>
+      </c>
+      <c r="D15">
+        <v>5531</v>
+      </c>
+      <c r="E15">
+        <v>110</v>
+      </c>
+      <c r="G15">
+        <v>3342</v>
+      </c>
+      <c r="H15">
+        <v>9</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>26</v>
+      </c>
+      <c r="K15">
+        <v>19</v>
+      </c>
+      <c r="L15">
+        <v>18</v>
+      </c>
+      <c r="M15">
+        <v>10</v>
+      </c>
+      <c r="O15">
+        <v>8</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>108</v>
+      </c>
+      <c r="AE15" t="str">
+        <v>Parn LINE photo fe9dd0f63e63 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Apple &amp; Pear 8, Mangosteen Blended 1, Mangosteen Lychee Blended 4, Pomegranate 1, Grape 4 | CHECK: items 8874 vs total sales 8873 (+1)</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>15/10/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C16">
+        <v>5667</v>
+      </c>
+      <c r="D16">
+        <v>4202</v>
+      </c>
+      <c r="E16">
+        <v>110</v>
+      </c>
+      <c r="G16">
+        <v>1465</v>
+      </c>
+      <c r="H16">
+        <v>9</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>7</v>
+      </c>
+      <c r="K16">
+        <v>13</v>
+      </c>
+      <c r="L16">
+        <v>18</v>
+      </c>
+      <c r="M16">
+        <v>3</v>
+      </c>
+      <c r="O16">
+        <v>4</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>68</v>
+      </c>
+      <c r="AE16" t="str">
+        <v>Parn LINE photo f918b3f949df (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Pear 4, Mangosteen Lychee Blended 4, Pomegranate 5, Grape 1 | CHECK: items 5664 vs total sales 5667 (-3)</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>16/10/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C17">
+        <v>5672</v>
+      </c>
+      <c r="D17">
+        <v>4328</v>
+      </c>
+      <c r="E17">
+        <v>55</v>
+      </c>
+      <c r="G17">
+        <v>1344</v>
+      </c>
+      <c r="H17">
+        <v>11</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>12</v>
+      </c>
+      <c r="K17">
+        <v>4</v>
+      </c>
+      <c r="L17">
+        <v>14</v>
+      </c>
+      <c r="M17">
+        <v>4</v>
+      </c>
+      <c r="O17">
+        <v>7</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>65</v>
+      </c>
+      <c r="AE17" t="str">
+        <v>Parn LINE photo 75e2ab1664c2 (B3 Daily Shop Report), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 3, Mangosteen Lychee Blended 6, Volcano Mix Fruit 1, Pear 1, Grape 2 | CHECK: items 5617 vs total sales 5672 (-55)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>